<commit_message>
test: add new task 106 and verify ci path
</commit_message>
<xml_diff>
--- a/task_center/task_manager.xlsx
+++ b/task_center/task_manager.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="25">
   <si>
     <t>id</t>
   </si>
@@ -96,6 +96,12 @@
   </si>
   <si>
     <t>develop</t>
+  </si>
+  <si>
+    <t>cicd测试01</t>
+  </si>
+  <si>
+    <t>ywkk667</t>
   </si>
 </sst>
 </file>
@@ -1294,8 +1300,8 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:N3"/>
-  <sheetFormatPr defaultColWidth="7.375" defaultRowHeight="13.5" outlineLevelRow="2"/>
+  <dimension ref="A1:N4"/>
+  <sheetFormatPr defaultColWidth="7.375" defaultRowHeight="13.5" outlineLevelRow="3"/>
   <cols>
     <col min="1" max="14" width="15.375" customWidth="1"/>
     <col min="15" max="16384" width="7.375" customWidth="1"/>
@@ -1409,6 +1415,38 @@
       <c r="M3" s="4"/>
       <c r="N3" s="4"/>
     </row>
+    <row r="4" ht="15" spans="1:14">
+      <c r="A4" s="2">
+        <v>106</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D4" s="2"/>
+      <c r="E4" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G4" s="2"/>
+      <c r="H4" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="J4" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="K4" s="1"/>
+      <c r="L4" s="1"/>
+      <c r="M4" s="4"/>
+      <c r="N4" s="4"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>

</xml_diff>